<commit_message>
Add read_context_xlsx and read_context_file; extend fixture with context questions
- Extended make_xlsx_fixture.R mapper with Q4/Q5 (interest before/after course)
  and added matching raw data columns; regenerated TEST101-01_FALL25.xlsx
- Appended read_context_xlsx (decodes XLSX numeric codes via CONTEXT_QUESTIONS)
  and read_context_file (dispatches on extension) to R/helpers.R
- Added two new tests: XLSX context decode (Low=2/Medium=2/High=3) and
  extension dispatch; all 15 tests pass
</commit_message>
<xml_diff>
--- a/tests/testthat/fixtures/TEST101-01_FALL25.xlsx
+++ b/tests/testthat/fixtures/TEST101-01_FALL25.xlsx
@@ -352,7 +352,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -401,6 +401,16 @@
           <t>Question 3</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Question 4</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Question 5</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -442,6 +452,16 @@
           <t>2</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -483,6 +503,16 @@
           <t>3</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -524,6 +554,16 @@
           <t>4</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -558,6 +598,16 @@
       <c r="I5" t="inlineStr">
         <is>
           <t>1</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -568,7 +618,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -619,6 +669,30 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Question 4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Course Interest and Demands - My interest in subject before course</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Question 5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Course Interest and Demands - My interest in subject after course</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix read_context_xlsx to strip trailing period so real XLSX context questions match; restore realistic fixture and add regression guard
</commit_message>
<xml_diff>
--- a/tests/testthat/fixtures/TEST101-01_FALL25.xlsx
+++ b/tests/testthat/fixtures/TEST101-01_FALL25.xlsx
@@ -677,7 +677,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Course Interest and Demands - My interest in subject before course</t>
+          <t>Course Interest and Demands - My interest in subject before course.</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Course Interest and Demands - My interest in subject after course</t>
+          <t>Course Interest and Demands - My interest in subject after course.</t>
         </is>
       </c>
     </row>

</xml_diff>